<commit_message>
data(employees, availability): extract 26 employees from av.xlsx
scripts/extract_from_av.py reads worker_templates/av.xlsx and writes
both canonical templates from scratch.

employees.xlsx — 26 rows:
  • numbers: 2000..2025 (sequential placeholder; real numbers TBD)
  • phones: 1234<num> (placeholder pattern; real numbers TBD)
  • professions (extracted from group headers in av.xlsx):
      קצינים  (2)
      מכונאות (6)
      בק״ש    (3)
      חשמל    (2)
      צריח    (1)
      חילוץ   (2)
      רכב     (5)
      נשק     (3)
      א.נ.ם   (2)
  • permissions: all technician (no info to distinguish)

employee_availability.xlsx — 26 × 73 days (01/05..12/07):
  • Mapped Hebrew status words to V/X:
      V: נוכח, נוכח - פתיחת צו, התארגנות, סגירת צו, סבב א/ב,
         יום ראשון, holiday names, names (substitutions), empty
      X: בית, אילוץ, צו סגור, אילוץ - צו סגור, "-"
  • Result: 1757 V + 141 X across 1898 cells.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/worker_templates/employees.xlsx
+++ b/worker_templates/employees.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,10 +29,6 @@
     <font>
       <b val="1"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00888888"/>
     </font>
     <font>
       <b val="1"/>
@@ -65,13 +61,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -440,13 +435,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -478,117 +473,650 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1001</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>נועה ברק</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>050-1110001</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>manager</t>
+      <c r="A2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>דור קריקב</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>12342000</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>קצינים</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>technician</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>1002</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>אבי כהן</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>050-1110002</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>warehouse</t>
+      <c r="A3" t="n">
+        <v>2001</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>לאון בניאס</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>12342001</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>קצינים</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>technician</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>1003</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>יואב לוי</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>050-1110003</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="A4" t="n">
+        <v>2002</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>בן ברקמן</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>12342002</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>מכונאות</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>דניס בולבינוב</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>12342003</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>מכונאות</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>משה בנעזרי</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>12342004</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>מכונאות</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ראזי אבו עביד</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>12342005</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>מכונאות</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>גלעד גבאי</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>12342006</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>מכונאות</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>מיכאל שבצנקו</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>12342007</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>מכונאות</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>שחף ניסים</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>12342008</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>בק״ש</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>אלכסנדר לויצקי</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>12342009</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>בק״ש</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>קיריל צ׳ורקוב</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>12342010</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>בק״ש</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2011</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>דמיטרי איטקין</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>12342011</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>חשמל</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>משה שכטר</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>12342012</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>חשמל</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>אלמוג כהן</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>12342013</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>צריח</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>רוני ביאנה</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>12342014</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>חילוץ</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>אלכסיי גרינברג</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>12342015</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>חילוץ</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>מקסים פלומבויים</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>12342016</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
         <is>
           <t>רכב</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>technician</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>1004</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>שרון ישראלי</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>050-1110004</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>חשמל</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>technician</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>1005</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>דנה אברהם</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>050-1110005</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>אופטיקה</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>2017</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ירין דוד</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>12342017</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>פואד אבו עאסי</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>12342018</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>דניאל קורולקוב</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>12342019</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>טל אסטרין</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>12342020</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>רכב</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>משה זלקה</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>12342021</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>נשק</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>יוני זנה</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>12342022</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>נשק</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ניתאי מלכה</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>12342023</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>נשק</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>סרגיי צירלוב</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>12342024</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>א.נ.ם</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>תומר סיגלוב</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>12342025</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>א.נ.ם</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>technician</t>
         </is>
@@ -605,99 +1133,68 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>הוראות מילוי</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>טבלה זו ממלאת את רשימת העובדים במערכת.</t>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>טבלת עובדים — חולץ מתוך av.xlsx (רשימת אנשי מקצוע + זמינות).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>כל עובד בשורה נפרדת.</t>
-        </is>
-      </c>
+      <c r="A4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr"/>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>עמודות:</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>עמודות:</t>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • מספר עובד — מספר רץ החל מ-2000 (הערך האמיתי יוחלף בעתיד).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • מספר עובד — מספר שלם וייחודי. משמש לכניסה למערכת. דוגמה: 1003.</t>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • שם — שם מלא, חולץ מ-av.xlsx.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • שם — שם מלא בעברית.</t>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • טלפון — placeholder בפורמט 1234&lt;מס׳ עובד&gt; עד שיגיעו מספרים אמיתיים.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • טלפון — מומלץ בפורמט 050-XXXXXXX. רשות (אבל מומלץ — משמש לכפתורי התקשרות ו-WhatsApp במערכת).</t>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • מקצוע — קבוצת המקצוע מ-av.xlsx (קצינים, מכונאות, בק״ש, חשמל, צריח, חילוץ, רכב, נשק, א.נ.ם).</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • מקצוע — שם המקצוע של העובד. רלוונטי בעיקר לטכנאים. אופציונלי. דוגמאות: "רכב", "חשמל", "אופטיקה".</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • הרשאה — אחת משלוש: technician (טכנאי, ברירת מחדל) / warehouse (מחסנאי) / manager (מנהל).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>הערות:</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • השורות שמופיעות באקסל הזה בצבע אפור הן דוגמאות — אפשר למחוק אותן ולהזין נתונים אמיתיים.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • רשימת המקצועות הסופית תיגזר אוטומטית מהערכים שתכתב בעמודת "מקצוע". אין צורך להגדיר מקצועות מראש.</t>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • הרשאה — כל העובדים סווגו זמנית כ-technician. נעדכן ידנית למנהל/מחסנאי בעתיד.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data(employees): map א.נ.ם to מחסנאי + warehouse permission
Per user clarification, א.נ.ם is the warehouse role, not a tank
specialty. Updated PROFESSION_MAP accordingly. Also refactored the
permissions assignment so it derives from the canonical profession
via PERMISSIONS_BY_PROFESSION (מנהל→manager, מחסנאי→warehouse,
everything else→technician).

Result:
  טנק:    14
  רכב:     5
  נשק:     3
  מנהל:    2  (manager)
  מחסנאי:  2  (warehouse) — סרגיי צירלוב, תומר סיגלוב

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/worker_templates/employees.xlsx
+++ b/worker_templates/employees.xlsx
@@ -1088,12 +1088,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>טנק</t>
+          <t>מחסנאי</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>technician</t>
+          <t>warehouse</t>
         </is>
       </c>
     </row>
@@ -1113,12 +1113,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>טנק</t>
+          <t>מחסנאי</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>technician</t>
+          <t>warehouse</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1211,26 +1211,33 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • קצינים → מנהל (גם הרשאה manager)</t>
+          <t xml:space="preserve">  • קצינים → מנהל   (הרשאה: manager)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • מכונאות / בק״ש / חשמל / צריח / חילוץ / א.נ.ם → טנק</t>
+          <t xml:space="preserve">  • א.נ.ם   → מחסנאי (הרשאה: warehouse)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • רכב → רכב</t>
+          <t xml:space="preserve">  • מכונאות / בק״ש / חשמל / צריח / חילוץ → טנק</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • רכב → רכב</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  • נשק → נשק</t>
         </is>

</xml_diff>

<commit_message>
data(employees): wire real employee numbers + phones (provided 2026-05-04)
Replaced the 2000-2025 placeholder numbers and 1234<num> placeholder
phones in extract_from_av.py with actual values per the user's roster.
Also added a NAME_OVERRIDE map: 'גלעד גבאי' (av.xlsx) is rendered as
'גילעד גבאי' (preferred display).

Re-ran extract_from_av.py → regenerated employees.xlsx and
employee_availability.xlsx with the new numbers.
Re-ran import_all.py → wiped & reloaded the DB:
  professions:            5
  employees:             26   (numbers 5108573..9999999)
  vehicles:              40
  employee_availability:572
Parts (1214) untouched.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/worker_templates/employees.xlsx
+++ b/worker_templates/employees.xlsx
@@ -474,71 +474,71 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2000</v>
+        <v>5108573</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>דור קריקב</t>
+          <t>מקסים פלומבויים</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>12342000</t>
+          <t>546505950</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>מנהל</t>
+          <t>רכב</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>manager</t>
+          <t>technician</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2001</v>
+        <v>5385987</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>לאון בניאס</t>
+          <t>אלכסיי גרינברג</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>12342001</t>
+          <t>532812908</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>מנהל</t>
+          <t>טנק</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>manager</t>
+          <t>technician</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2002</v>
+        <v>5754689</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>בן ברקמן</t>
+          <t>ניתאי מלכה</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>12342002</t>
+          <t>546526336</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>טנק</t>
+          <t>נשק</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -549,21 +549,21 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2003</v>
+        <v>5763399</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>דניס בולבינוב</t>
+          <t>יוני זנה</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>12342003</t>
+          <t>508123242</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>טנק</t>
+          <t>נשק</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -574,21 +574,21 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2004</v>
+        <v>6134018</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>משה בנעזרי</t>
+          <t>פואד אבו עאסי</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>12342004</t>
+          <t>543932707</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>טנק</t>
+          <t>רכב</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -599,16 +599,16 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2005</v>
+        <v>6891337</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ראזי אבו עביד</t>
+          <t>רוני ביאנה</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>12342005</t>
+          <t>528400558</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -624,21 +624,21 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2006</v>
+        <v>7414543</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>גלעד גבאי</t>
+          <t>משה זלקה</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12342006</t>
+          <t>505168600</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>טנק</t>
+          <t>נשק</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -649,32 +649,32 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2007</v>
+        <v>7471311</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>מיכאל שבצנקו</t>
+          <t>סרגיי צירלוב</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12342007</t>
+          <t>526230535</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>טנק</t>
+          <t>מחסנאי</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>technician</t>
+          <t>warehouse</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2008</v>
+        <v>7548287</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -683,7 +683,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12342008</t>
+          <t>504380030</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -699,16 +699,16 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2009</v>
+        <v>7600591</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>אלכסנדר לויצקי</t>
+          <t>משה בנעזרי</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>12342009</t>
+          <t>508080543</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -724,16 +724,16 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>2010</v>
+        <v>7667042</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>קיריל צ׳ורקוב</t>
+          <t>דניס בולבינוב</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12342010</t>
+          <t>546458538</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -749,41 +749,41 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2011</v>
+        <v>7777777</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>דמיטרי איטקין</t>
+          <t>תומר סיגלוב</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>12342011</t>
+          <t>536201993</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>טנק</t>
+          <t>מחסנאי</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>technician</t>
+          <t>warehouse</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>2012</v>
+        <v>8048029</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>משה שכטר</t>
+          <t>בן ברקמן</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>12342012</t>
+          <t>526411633</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -799,21 +799,21 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>2013</v>
+        <v>8141927</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>אלמוג כהן</t>
+          <t>דניאל קורולקוב</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>12342013</t>
+          <t>502798896</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>טנק</t>
+          <t>רכב</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -824,21 +824,21 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>2014</v>
+        <v>8169903</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>רוני ביאנה</t>
+          <t>טל אסטרין</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>12342014</t>
+          <t>508120175</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>טנק</t>
+          <t>רכב</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -849,16 +849,16 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>2015</v>
+        <v>8183890</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>אלכסיי גרינברג</t>
+          <t>אלמוג כהן</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>12342015</t>
+          <t>542299927</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -874,16 +874,16 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>2016</v>
+        <v>8190085</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>מקסים פלומבויים</t>
+          <t>ירין דוד</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>12342016</t>
+          <t>504647481</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -899,21 +899,21 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2017</v>
+        <v>8266875</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ירין דוד</t>
+          <t>מיכאל שבצנקו</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>12342017</t>
+          <t>507288003</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>רכב</t>
+          <t>טנק</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -924,46 +924,46 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>2018</v>
+        <v>8275186</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>פואד אבו עאסי</t>
+          <t>דור קריקב</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>12342018</t>
+          <t>505580129</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>רכב</t>
+          <t>מנהל</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>technician</t>
+          <t>manager</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>2019</v>
+        <v>8451889</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>דניאל קורולקוב</t>
+          <t>דמיטרי איטקין</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>12342019</t>
+          <t>526354188</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>רכב</t>
+          <t>טנק</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -974,21 +974,21 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>2020</v>
+        <v>8592587</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>טל אסטרין</t>
+          <t>ראזי אבו עביד</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>12342020</t>
+          <t>523119258</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>רכב</t>
+          <t>טנק</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -999,21 +999,21 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>2021</v>
+        <v>8831115</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>משה זלקה</t>
+          <t>קיריל צ׳ורקוב</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>12342021</t>
+          <t>1234</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>נשק</t>
+          <t>טנק</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1024,21 +1024,21 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>2022</v>
+        <v>8840972</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>יוני זנה</t>
+          <t>אלכסנדר לויצקי</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>12342022</t>
+          <t>529579147</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>נשק</t>
+          <t>טנק</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1049,21 +1049,21 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>2023</v>
+        <v>9014610</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ניתאי מלכה</t>
+          <t>גילעד גבאי</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>12342023</t>
+          <t>542040911</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>נשק</t>
+          <t>טנק</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1074,51 +1074,51 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>2024</v>
+        <v>9175267</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>סרגיי צירלוב</t>
+          <t>משה שכטר</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>12342024</t>
+          <t>5678</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>מחסנאי</t>
+          <t>טנק</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>warehouse</t>
+          <t>technician</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>2025</v>
+        <v>9999999</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>תומר סיגלוב</t>
+          <t>לאון בניאס</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>12342025</t>
+          <t>502880886</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>מחסנאי</t>
+          <t>מנהל</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>warehouse</t>
+          <t>manager</t>
         </is>
       </c>
     </row>
@@ -1166,21 +1166,21 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • מספר עובד — מספר רץ החל מ-2000 (placeholder).</t>
+          <t xml:space="preserve">  • מספר עובד — מספר אישי אמיתי (מ-NAME_NUMBER ב-extract_from_av.py).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • שם — שם מלא, חולץ מ-av.xlsx.</t>
+          <t xml:space="preserve">  • שם — שם מלא, חולץ מ-av.xlsx (עם NAME_OVERRIDE לאיותים מועדפים).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • טלפון — placeholder בפורמט 1234&lt;מס׳ עובד&gt;.</t>
+          <t xml:space="preserve">  • טלפון — מספר טלפון אמיתי (מ-NAME_PHONE), עם נפילה ל-1234&lt;מס׳&gt; עבור עובדים שלא ניתן להם מספר.</t>
         </is>
       </c>
     </row>

</xml_diff>